<commit_message>
P_aux calculated is now saved in the output h5 file
</commit_message>
<xml_diff>
--- a/outputs/compare_tseeded_lump_t_startup.xlsx
+++ b/outputs/compare_tseeded_lump_t_startup.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="All_Results" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ddstartup_20251111_220719_param" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ddstartup_20251112_105650_param" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="ddstartup_20251111_232630_param" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="S_Q1_Best" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="S_Q1_Median" sheetId="6" state="visible" r:id="rId6"/>
@@ -494,7 +494,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -514,16 +514,16 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>652794.8476254502</v>
+        <v>652748.5472934669</v>
       </c>
       <c r="G2" t="n">
-        <v>652794.8476254502</v>
+        <v>652748.5472934669</v>
       </c>
       <c r="H2" t="n">
-        <v>652794.8476254502</v>
+        <v>652748.5472934669</v>
       </c>
       <c r="I2" t="n">
-        <v>652794.8476254502</v>
+        <v>652748.5472934669</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -532,7 +532,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -552,16 +552,16 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>4360994.697124124</v>
+        <v>4315890.926647455</v>
       </c>
       <c r="G3" t="n">
-        <v>4360994.697124124</v>
+        <v>4315890.926647455</v>
       </c>
       <c r="H3" t="n">
-        <v>4360994.697124124</v>
+        <v>4315890.926647455</v>
       </c>
       <c r="I3" t="n">
-        <v>4360994.697124124</v>
+        <v>4315890.926647455</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -570,7 +570,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -590,16 +590,16 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>8289794.985555269</v>
+        <v>8165327.087865899</v>
       </c>
       <c r="G4" t="n">
-        <v>8289794.985555269</v>
+        <v>8165327.087865899</v>
       </c>
       <c r="H4" t="n">
-        <v>8289794.985555269</v>
+        <v>8165327.087865899</v>
       </c>
       <c r="I4" t="n">
-        <v>8289794.985555269</v>
+        <v>8165327.087865899</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -608,7 +608,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -628,16 +628,16 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>13989385.84561866</v>
+        <v>13768415.33543325</v>
       </c>
       <c r="G5" t="n">
-        <v>13989385.84561866</v>
+        <v>13768415.33543325</v>
       </c>
       <c r="H5" t="n">
-        <v>13989385.84561866</v>
+        <v>13768415.33543325</v>
       </c>
       <c r="I5" t="n">
-        <v>13989385.84561866</v>
+        <v>13768415.33543325</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -646,7 +646,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -666,16 +666,16 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>24035722.23546692</v>
+        <v>23468644.95781989</v>
       </c>
       <c r="G6" t="n">
-        <v>24035722.23546692</v>
+        <v>23468644.95781989</v>
       </c>
       <c r="H6" t="n">
-        <v>24035722.23546692</v>
+        <v>23468644.95781989</v>
       </c>
       <c r="I6" t="n">
-        <v>24035722.23546692</v>
+        <v>23468644.95781989</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -684,7 +684,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -704,16 +704,16 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>38678460.78115635</v>
+        <v>37731993.46921755</v>
       </c>
       <c r="G7" t="n">
-        <v>38678460.78115635</v>
+        <v>37731993.46921755</v>
       </c>
       <c r="H7" t="n">
-        <v>38678460.78115635</v>
+        <v>37731993.46921755</v>
       </c>
       <c r="I7" t="n">
-        <v>38678460.78115635</v>
+        <v>37731993.46921755</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -722,7 +722,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -742,16 +742,16 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>67569956.49294126</v>
+        <v>66614453.37517199</v>
       </c>
       <c r="G8" t="n">
-        <v>67569956.49294126</v>
+        <v>66614453.37517199</v>
       </c>
       <c r="H8" t="n">
-        <v>67569956.49294126</v>
+        <v>66614453.37517199</v>
       </c>
       <c r="I8" t="n">
-        <v>67569956.49294126</v>
+        <v>66614453.37517199</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -760,7 +760,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -780,16 +780,16 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>129798926.3929557</v>
+        <v>128233856.3830587</v>
       </c>
       <c r="G9" t="n">
-        <v>129798926.3929557</v>
+        <v>128233856.3830587</v>
       </c>
       <c r="H9" t="n">
-        <v>129798926.3929557</v>
+        <v>128233856.3830587</v>
       </c>
       <c r="I9" t="n">
-        <v>129798926.3929557</v>
+        <v>128233856.3830587</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -1266,26 +1266,30 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1564918087945841</v>
+        <v>229854446620483.7</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>434516298.6625866</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+        <v>94627993.93096329</v>
+      </c>
+      <c r="G2" t="n">
+        <v>32719896.78044747</v>
+      </c>
+      <c r="H2" t="n">
+        <v>32719896.78044747</v>
+      </c>
       <c r="I2" t="n">
-        <v>1.794216891916112</v>
+        <v>1.650867848440599</v>
       </c>
       <c r="J2" t="n">
-        <v>3.223538284107875</v>
+        <v>2.892062727640095</v>
       </c>
       <c r="K2" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
         <v>1.05</v>
@@ -1297,7 +1301,7 @@
         <v>100</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -1308,11 +1312,11 @@
         <v>0.3</v>
       </c>
       <c r="R2" t="n">
-        <v>24791</v>
+        <v>20738</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
-        <v>1.5e+20</v>
+        <v>7e+19</v>
       </c>
       <c r="U2" t="n">
         <v>1.111111111111111e-07</v>
@@ -1321,7 +1325,7 @@
         <v>1</v>
       </c>
       <c r="W2" t="n">
-        <v>38678460.78115635</v>
+        <v>37731993.46921755</v>
       </c>
       <c r="X2" t="n">
         <v>14400</v>
@@ -1331,10 +1335,10 @@
       </c>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AB2" t="n">
-        <v>173879787.5495379</v>
+        <v>25539382.95783152</v>
       </c>
     </row>
     <row r="3">
@@ -1592,35 +1596,39 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.941232953524845e+16</v>
+        <v>4.549410069975693e+16</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1495403908.526144</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+        <v>3862367099.222991</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6485370276.752956</v>
+      </c>
+      <c r="H2" t="n">
+        <v>6485370276.752956</v>
+      </c>
       <c r="I2" t="n">
-        <v>0.1082164820307202</v>
+        <v>0.303034938572553</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2320538920857703</v>
+        <v>0.5955507448923596</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="L2" t="n">
-        <v>1.3</v>
+        <v>1.15</v>
       </c>
       <c r="M2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N2" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="O2" t="n">
         <v>0.9</v>
@@ -1634,11 +1642,11 @@
         <v>0.4</v>
       </c>
       <c r="R2" t="n">
-        <v>141316</v>
+        <v>82312</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
-        <v>7e+19</v>
+        <v>2e+20</v>
       </c>
       <c r="U2" t="n">
         <v>6.944444444444444e-08</v>
@@ -1647,20 +1655,20 @@
         <v>1</v>
       </c>
       <c r="W2" t="n">
-        <v>67569956.49294126</v>
+        <v>66614453.37517199</v>
       </c>
       <c r="X2" t="n">
         <v>14400</v>
       </c>
       <c r="Y2" t="n">
-        <v>86400</v>
+        <v>7200</v>
       </c>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="n">
         <v>0.1</v>
       </c>
       <c r="AB2" t="n">
-        <v>1348078439.947809</v>
+        <v>3159312548.594231</v>
       </c>
     </row>
     <row r="3">
@@ -1918,38 +1926,42 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2.849988870111725e+16</v>
+        <v>2.402685011474862e+17</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1892559878.619266</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+        <v>24414757690.22276</v>
+      </c>
+      <c r="G2" t="n">
+        <v>33800133133.8574</v>
+      </c>
+      <c r="H2" t="n">
+        <v>33800133133.8574</v>
+      </c>
       <c r="I2" t="n">
-        <v>1.649362497079111</v>
+        <v>0.3527676829111169</v>
       </c>
       <c r="J2" t="n">
-        <v>2.892062727640095</v>
+        <v>0.7223272640238992</v>
       </c>
       <c r="K2" t="n">
         <v>0.5</v>
       </c>
       <c r="L2" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
       <c r="M2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="N2" t="n">
         <v>2000</v>
       </c>
       <c r="O2" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -1960,33 +1972,33 @@
         <v>0.3</v>
       </c>
       <c r="R2" t="n">
-        <v>177990</v>
+        <v>204734</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
-        <v>7e+19</v>
+        <v>2e+20</v>
       </c>
       <c r="U2" t="n">
-        <v>2.777777777777778e-08</v>
+        <v>1.111111111111111e-07</v>
       </c>
       <c r="V2" t="b">
         <v>1</v>
       </c>
       <c r="W2" t="n">
-        <v>129798926.3929557</v>
+        <v>128233856.3830587</v>
       </c>
       <c r="X2" t="n">
         <v>43200</v>
       </c>
       <c r="Y2" t="n">
-        <v>7200</v>
+        <v>43200</v>
       </c>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="AB2" t="n">
-        <v>791663575.0310347</v>
+        <v>26696500127.49847</v>
       </c>
     </row>
     <row r="3">
@@ -2341,18 +2353,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1416255352099782</v>
+        <v>3403313122315846</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>24414757690.22276</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
@@ -2368,7 +2384,7 @@
         <v>2000</v>
       </c>
       <c r="P3" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -2376,10 +2392,10 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="S3" t="n">
-        <v>209792</v>
+        <v>209807</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="n">
@@ -2392,7 +2408,7 @@
         <v>1</v>
       </c>
       <c r="X3" t="n">
-        <v>652794.8476254502</v>
+        <v>652748.5472934669</v>
       </c>
       <c r="Y3" t="n">
         <v>14400</v>
@@ -2405,7 +2421,7 @@
         <v>5</v>
       </c>
       <c r="AC3" t="n">
-        <v>157361705.7888646</v>
+        <v>378145902.4795384</v>
       </c>
     </row>
     <row r="4">
@@ -2511,31 +2527,35 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>5091186253411937</v>
+        <v>705390119754817</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>6866650600.375151</v>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+        <v>1220737884.511138</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>0.75</v>
       </c>
       <c r="M5" t="n">
-        <v>1.15</v>
+        <v>1.05</v>
       </c>
       <c r="N5" t="n">
         <v>20</v>
       </c>
       <c r="O5" t="n">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="P5" t="n">
         <v>0.9</v>
@@ -2546,36 +2566,36 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="S5" t="n">
-        <v>150945</v>
+        <v>51271</v>
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="n">
-        <v>1.5e+20</v>
+        <v>2e+20</v>
       </c>
       <c r="V5" t="n">
-        <v>2.777777777777778e-08</v>
+        <v>6.944444444444444e-08</v>
       </c>
       <c r="W5" t="b">
         <v>1</v>
       </c>
       <c r="X5" t="n">
-        <v>4360994.697124124</v>
+        <v>4315890.926647455</v>
       </c>
       <c r="Y5" t="n">
+        <v>21600</v>
+      </c>
+      <c r="Z5" t="n">
         <v>43200</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>7200</v>
       </c>
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="n">
         <v>5</v>
       </c>
       <c r="AC5" t="n">
-        <v>141421840.3725538</v>
+        <v>48985424.9829734</v>
       </c>
     </row>
     <row r="6">
@@ -2683,22 +2703,26 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1020416278073986</v>
+        <v>3144972497151465</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>747701954.2630719</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+        <v>6103689422.55569</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M7" t="n">
         <v>1.05</v>
@@ -2710,7 +2734,7 @@
         <v>500</v>
       </c>
       <c r="P7" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -2718,36 +2742,36 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="S7" t="n">
-        <v>91925</v>
+        <v>102384</v>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="n">
-        <v>7e+19</v>
+        <v>2e+20</v>
       </c>
       <c r="V7" t="n">
-        <v>1.111111111111111e-07</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="W7" t="b">
         <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>8289794.985555269</v>
+        <v>8165327.087865899</v>
       </c>
       <c r="Y7" t="n">
-        <v>21600</v>
+        <v>14400</v>
       </c>
       <c r="Z7" t="n">
         <v>7200</v>
       </c>
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC7" t="n">
-        <v>113379586.4526651</v>
+        <v>87360347.14309625</v>
       </c>
     </row>
     <row r="8">
@@ -2853,31 +2877,35 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>5165519965489169</v>
+        <v>272270365750398</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>2172581493.312933</v>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+        <v>94627993.93096329</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>0.5</v>
       </c>
       <c r="M9" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
       <c r="N9" t="n">
         <v>15</v>
       </c>
       <c r="O9" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="P9" t="n">
         <v>0.9</v>
@@ -2891,11 +2919,11 @@
         <v>0.4</v>
       </c>
       <c r="S9" t="n">
-        <v>80333</v>
+        <v>22499</v>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="n">
-        <v>1.5e+20</v>
+        <v>7e+19</v>
       </c>
       <c r="V9" t="n">
         <v>1.111111111111111e-07</v>
@@ -2904,7 +2932,7 @@
         <v>1</v>
       </c>
       <c r="X9" t="n">
-        <v>13989385.84561866</v>
+        <v>13768415.33543325</v>
       </c>
       <c r="Y9" t="n">
         <v>43200</v>
@@ -2917,7 +2945,7 @@
         <v>5</v>
       </c>
       <c r="AC9" t="n">
-        <v>573946662.8321298</v>
+        <v>30252262.86115533</v>
       </c>
     </row>
     <row r="10">
@@ -3025,35 +3053,35 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3761915752841065</v>
+        <v>735678291552867.6</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>1601740505.970906</v>
-      </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="n">
-        <v>1.262886935408163</v>
-      </c>
-      <c r="K11" t="n">
-        <v>2.361895677493635</v>
-      </c>
+        <v>320348101.1941811</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="M11" t="n">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="N11" t="n">
         <v>10</v>
       </c>
       <c r="O11" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="P11" t="n">
         <v>0.7</v>
@@ -3067,33 +3095,33 @@
         <v>0.3</v>
       </c>
       <c r="S11" t="n">
-        <v>66766</v>
+        <v>16167</v>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="n">
         <v>2e+20</v>
       </c>
       <c r="V11" t="n">
-        <v>6.944444444444444e-08</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="W11" t="b">
         <v>1</v>
       </c>
       <c r="X11" t="n">
-        <v>24035722.23546692</v>
+        <v>23468644.95781989</v>
       </c>
       <c r="Y11" t="n">
-        <v>14400</v>
+        <v>43200</v>
       </c>
       <c r="Z11" t="n">
         <v>43200</v>
       </c>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="AC11" t="n">
-        <v>261244149.5028517</v>
+        <v>20435508.09869077</v>
       </c>
     </row>
     <row r="12">
@@ -3110,26 +3138,30 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1564918087945841</v>
+        <v>229854446620483.7</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>434516298.6625866</v>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+        <v>94627993.93096329</v>
+      </c>
+      <c r="H12" t="n">
+        <v>32719896.78044747</v>
+      </c>
+      <c r="I12" t="n">
+        <v>32719896.78044747</v>
+      </c>
       <c r="J12" t="n">
-        <v>1.794216891916112</v>
+        <v>1.650867848440599</v>
       </c>
       <c r="K12" t="n">
-        <v>3.223538284107875</v>
+        <v>2.892062727640095</v>
       </c>
       <c r="L12" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M12" t="n">
         <v>1.05</v>
@@ -3141,7 +3173,7 @@
         <v>100</v>
       </c>
       <c r="P12" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -3152,11 +3184,11 @@
         <v>0.3</v>
       </c>
       <c r="S12" t="n">
-        <v>24791</v>
+        <v>20738</v>
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="n">
-        <v>1.5e+20</v>
+        <v>7e+19</v>
       </c>
       <c r="V12" t="n">
         <v>1.111111111111111e-07</v>
@@ -3165,7 +3197,7 @@
         <v>1</v>
       </c>
       <c r="X12" t="n">
-        <v>38678460.78115635</v>
+        <v>37731993.46921755</v>
       </c>
       <c r="Y12" t="n">
         <v>14400</v>
@@ -3175,10 +3207,10 @@
       </c>
       <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AC12" t="n">
-        <v>173879787.5495379</v>
+        <v>25539382.95783152</v>
       </c>
     </row>
     <row r="13">
@@ -3286,35 +3318,39 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1.941232953524845e+16</v>
+        <v>4.549410069975693e+16</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>1495403908.526144</v>
-      </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
+        <v>3862367099.222991</v>
+      </c>
+      <c r="H14" t="n">
+        <v>6485370276.752956</v>
+      </c>
+      <c r="I14" t="n">
+        <v>6485370276.752956</v>
+      </c>
       <c r="J14" t="n">
-        <v>0.1082164820307202</v>
+        <v>0.303034938572553</v>
       </c>
       <c r="K14" t="n">
-        <v>0.2320538920857703</v>
+        <v>0.5955507448923596</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="M14" t="n">
-        <v>1.3</v>
+        <v>1.15</v>
       </c>
       <c r="N14" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="O14" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="P14" t="n">
         <v>0.9</v>
@@ -3328,11 +3364,11 @@
         <v>0.4</v>
       </c>
       <c r="S14" t="n">
-        <v>141316</v>
+        <v>82312</v>
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="n">
-        <v>7e+19</v>
+        <v>2e+20</v>
       </c>
       <c r="V14" t="n">
         <v>6.944444444444444e-08</v>
@@ -3341,20 +3377,20 @@
         <v>1</v>
       </c>
       <c r="X14" t="n">
-        <v>67569956.49294126</v>
+        <v>66614453.37517199</v>
       </c>
       <c r="Y14" t="n">
         <v>14400</v>
       </c>
       <c r="Z14" t="n">
-        <v>86400</v>
+        <v>7200</v>
       </c>
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="n">
         <v>0.1</v>
       </c>
       <c r="AC14" t="n">
-        <v>1348078439.947809</v>
+        <v>3159312548.594231</v>
       </c>
     </row>
     <row r="15">
@@ -3462,38 +3498,42 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>2.849988870111725e+16</v>
+        <v>2.402685011474862e+17</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>1892559878.619266</v>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
+        <v>24414757690.22276</v>
+      </c>
+      <c r="H16" t="n">
+        <v>33800133133.8574</v>
+      </c>
+      <c r="I16" t="n">
+        <v>33800133133.8574</v>
+      </c>
       <c r="J16" t="n">
-        <v>1.649362497079111</v>
+        <v>0.3527676829111169</v>
       </c>
       <c r="K16" t="n">
-        <v>2.892062727640095</v>
+        <v>0.7223272640238992</v>
       </c>
       <c r="L16" t="n">
         <v>0.5</v>
       </c>
       <c r="M16" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
       <c r="N16" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="O16" t="n">
         <v>2000</v>
       </c>
       <c r="P16" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -3504,33 +3544,33 @@
         <v>0.3</v>
       </c>
       <c r="S16" t="n">
-        <v>177990</v>
+        <v>204734</v>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="n">
-        <v>7e+19</v>
+        <v>2e+20</v>
       </c>
       <c r="V16" t="n">
-        <v>2.777777777777778e-08</v>
+        <v>1.111111111111111e-07</v>
       </c>
       <c r="W16" t="b">
         <v>1</v>
       </c>
       <c r="X16" t="n">
-        <v>129798926.3929557</v>
+        <v>128233856.3830587</v>
       </c>
       <c r="Y16" t="n">
         <v>43200</v>
       </c>
       <c r="Z16" t="n">
-        <v>7200</v>
+        <v>43200</v>
       </c>
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="AC16" t="n">
-        <v>791663575.0310347</v>
+        <v>26696500127.49847</v>
       </c>
     </row>
     <row r="17">
@@ -3791,18 +3831,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1416255352099782</v>
+        <v>3403313122315846</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
         <v>24414757690.22276</v>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
@@ -3818,7 +3862,7 @@
         <v>2000</v>
       </c>
       <c r="O2" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -3826,10 +3870,10 @@
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="R2" t="n">
-        <v>209792</v>
+        <v>209807</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
@@ -3842,7 +3886,7 @@
         <v>1</v>
       </c>
       <c r="W2" t="n">
-        <v>652794.8476254502</v>
+        <v>652748.5472934669</v>
       </c>
       <c r="X2" t="n">
         <v>14400</v>
@@ -3855,7 +3899,7 @@
         <v>5</v>
       </c>
       <c r="AB2" t="n">
-        <v>157361705.7888646</v>
+        <v>378145902.4795384</v>
       </c>
     </row>
     <row r="3">
@@ -3869,31 +3913,35 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5091186253411937</v>
+        <v>705390119754817</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>6866650600.375151</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+        <v>1220737884.511138</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
         <v>0.75</v>
       </c>
       <c r="L3" t="n">
-        <v>1.15</v>
+        <v>1.05</v>
       </c>
       <c r="M3" t="n">
         <v>20</v>
       </c>
       <c r="N3" t="n">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="O3" t="n">
         <v>0.9</v>
@@ -3904,36 +3952,36 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="R3" t="n">
-        <v>150945</v>
+        <v>51271</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
-        <v>1.5e+20</v>
+        <v>2e+20</v>
       </c>
       <c r="U3" t="n">
-        <v>2.777777777777778e-08</v>
+        <v>6.944444444444444e-08</v>
       </c>
       <c r="V3" t="b">
         <v>1</v>
       </c>
       <c r="W3" t="n">
-        <v>4360994.697124124</v>
+        <v>4315890.926647455</v>
       </c>
       <c r="X3" t="n">
+        <v>21600</v>
+      </c>
+      <c r="Y3" t="n">
         <v>43200</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>7200</v>
       </c>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="n">
         <v>5</v>
       </c>
       <c r="AB3" t="n">
-        <v>141421840.3725538</v>
+        <v>48985424.9829734</v>
       </c>
     </row>
     <row r="4">
@@ -3947,22 +3995,26 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1020416278073986</v>
+        <v>3144972497151465</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>747701954.2630719</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+        <v>6103689422.55569</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L4" t="n">
         <v>1.05</v>
@@ -3974,7 +4026,7 @@
         <v>500</v>
       </c>
       <c r="O4" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -3982,36 +4034,36 @@
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="R4" t="n">
-        <v>91925</v>
+        <v>102384</v>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
-        <v>7e+19</v>
+        <v>2e+20</v>
       </c>
       <c r="U4" t="n">
-        <v>1.111111111111111e-07</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="V4" t="b">
         <v>1</v>
       </c>
       <c r="W4" t="n">
-        <v>8289794.985555269</v>
+        <v>8165327.087865899</v>
       </c>
       <c r="X4" t="n">
-        <v>21600</v>
+        <v>14400</v>
       </c>
       <c r="Y4" t="n">
         <v>7200</v>
       </c>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AB4" t="n">
-        <v>113379586.4526651</v>
+        <v>87360347.14309625</v>
       </c>
     </row>
     <row r="5">
@@ -4025,31 +4077,35 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5165519965489169</v>
+        <v>272270365750398</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2172581493.312933</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+        <v>94627993.93096329</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
         <v>0.5</v>
       </c>
       <c r="L5" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
       <c r="M5" t="n">
         <v>15</v>
       </c>
       <c r="N5" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="O5" t="n">
         <v>0.9</v>
@@ -4063,11 +4119,11 @@
         <v>0.4</v>
       </c>
       <c r="R5" t="n">
-        <v>80333</v>
+        <v>22499</v>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
-        <v>1.5e+20</v>
+        <v>7e+19</v>
       </c>
       <c r="U5" t="n">
         <v>1.111111111111111e-07</v>
@@ -4076,7 +4132,7 @@
         <v>1</v>
       </c>
       <c r="W5" t="n">
-        <v>13989385.84561866</v>
+        <v>13768415.33543325</v>
       </c>
       <c r="X5" t="n">
         <v>43200</v>
@@ -4089,7 +4145,7 @@
         <v>5</v>
       </c>
       <c r="AB5" t="n">
-        <v>573946662.8321298</v>
+        <v>30252262.86115533</v>
       </c>
     </row>
     <row r="6">
@@ -4103,35 +4159,35 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3761915752841065</v>
+        <v>735678291552867.6</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1601740505.970906</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="n">
-        <v>1.262886935408163</v>
-      </c>
-      <c r="J6" t="n">
-        <v>2.361895677493635</v>
-      </c>
+        <v>320348101.1941811</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="M6" t="n">
         <v>10</v>
       </c>
       <c r="N6" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="O6" t="n">
         <v>0.7</v>
@@ -4145,33 +4201,33 @@
         <v>0.3</v>
       </c>
       <c r="R6" t="n">
-        <v>66766</v>
+        <v>16167</v>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="n">
         <v>2e+20</v>
       </c>
       <c r="U6" t="n">
-        <v>6.944444444444444e-08</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="V6" t="b">
         <v>1</v>
       </c>
       <c r="W6" t="n">
-        <v>24035722.23546692</v>
+        <v>23468644.95781989</v>
       </c>
       <c r="X6" t="n">
-        <v>14400</v>
+        <v>43200</v>
       </c>
       <c r="Y6" t="n">
         <v>43200</v>
       </c>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="AB6" t="n">
-        <v>261244149.5028517</v>
+        <v>20435508.09869077</v>
       </c>
     </row>
     <row r="7">
@@ -4185,26 +4241,30 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1564918087945841</v>
+        <v>229854446620483.7</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>434516298.6625866</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+        <v>94627993.93096329</v>
+      </c>
+      <c r="G7" t="n">
+        <v>32719896.78044747</v>
+      </c>
+      <c r="H7" t="n">
+        <v>32719896.78044747</v>
+      </c>
       <c r="I7" t="n">
-        <v>1.794216891916112</v>
+        <v>1.650867848440599</v>
       </c>
       <c r="J7" t="n">
-        <v>3.223538284107875</v>
+        <v>2.892062727640095</v>
       </c>
       <c r="K7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
         <v>1.05</v>
@@ -4216,7 +4276,7 @@
         <v>100</v>
       </c>
       <c r="O7" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -4227,11 +4287,11 @@
         <v>0.3</v>
       </c>
       <c r="R7" t="n">
-        <v>24791</v>
+        <v>20738</v>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
-        <v>1.5e+20</v>
+        <v>7e+19</v>
       </c>
       <c r="U7" t="n">
         <v>1.111111111111111e-07</v>
@@ -4240,7 +4300,7 @@
         <v>1</v>
       </c>
       <c r="W7" t="n">
-        <v>38678460.78115635</v>
+        <v>37731993.46921755</v>
       </c>
       <c r="X7" t="n">
         <v>14400</v>
@@ -4250,10 +4310,10 @@
       </c>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AB7" t="n">
-        <v>173879787.5495379</v>
+        <v>25539382.95783152</v>
       </c>
     </row>
     <row r="8">
@@ -4267,35 +4327,39 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.941232953524845e+16</v>
+        <v>4.549410069975693e+16</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>1495403908.526144</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+        <v>3862367099.222991</v>
+      </c>
+      <c r="G8" t="n">
+        <v>6485370276.752956</v>
+      </c>
+      <c r="H8" t="n">
+        <v>6485370276.752956</v>
+      </c>
       <c r="I8" t="n">
-        <v>0.1082164820307202</v>
+        <v>0.303034938572553</v>
       </c>
       <c r="J8" t="n">
-        <v>0.2320538920857703</v>
+        <v>0.5955507448923596</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="L8" t="n">
-        <v>1.3</v>
+        <v>1.15</v>
       </c>
       <c r="M8" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N8" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="O8" t="n">
         <v>0.9</v>
@@ -4309,11 +4373,11 @@
         <v>0.4</v>
       </c>
       <c r="R8" t="n">
-        <v>141316</v>
+        <v>82312</v>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="n">
-        <v>7e+19</v>
+        <v>2e+20</v>
       </c>
       <c r="U8" t="n">
         <v>6.944444444444444e-08</v>
@@ -4322,20 +4386,20 @@
         <v>1</v>
       </c>
       <c r="W8" t="n">
-        <v>67569956.49294126</v>
+        <v>66614453.37517199</v>
       </c>
       <c r="X8" t="n">
         <v>14400</v>
       </c>
       <c r="Y8" t="n">
-        <v>86400</v>
+        <v>7200</v>
       </c>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="n">
         <v>0.1</v>
       </c>
       <c r="AB8" t="n">
-        <v>1348078439.947809</v>
+        <v>3159312548.594231</v>
       </c>
     </row>
     <row r="9">
@@ -4349,38 +4413,42 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.849988870111725e+16</v>
+        <v>2.402685011474862e+17</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>1892559878.619266</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+        <v>24414757690.22276</v>
+      </c>
+      <c r="G9" t="n">
+        <v>33800133133.8574</v>
+      </c>
+      <c r="H9" t="n">
+        <v>33800133133.8574</v>
+      </c>
       <c r="I9" t="n">
-        <v>1.649362497079111</v>
+        <v>0.3527676829111169</v>
       </c>
       <c r="J9" t="n">
-        <v>2.892062727640095</v>
+        <v>0.7223272640238992</v>
       </c>
       <c r="K9" t="n">
         <v>0.5</v>
       </c>
       <c r="L9" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
       <c r="M9" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="N9" t="n">
         <v>2000</v>
       </c>
       <c r="O9" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -4391,33 +4459,33 @@
         <v>0.3</v>
       </c>
       <c r="R9" t="n">
-        <v>177990</v>
+        <v>204734</v>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
-        <v>7e+19</v>
+        <v>2e+20</v>
       </c>
       <c r="U9" t="n">
-        <v>2.777777777777778e-08</v>
+        <v>1.111111111111111e-07</v>
       </c>
       <c r="V9" t="b">
         <v>1</v>
       </c>
       <c r="W9" t="n">
-        <v>129798926.3929557</v>
+        <v>128233856.3830587</v>
       </c>
       <c r="X9" t="n">
         <v>43200</v>
       </c>
       <c r="Y9" t="n">
-        <v>7200</v>
+        <v>43200</v>
       </c>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="AB9" t="n">
-        <v>791663575.0310347</v>
+        <v>26696500127.49847</v>
       </c>
     </row>
   </sheetData>
@@ -5527,18 +5595,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1416255352099782</v>
+        <v>3403313122315846</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
         <v>24414757690.22276</v>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
@@ -5554,7 +5626,7 @@
         <v>2000</v>
       </c>
       <c r="O3" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -5562,10 +5634,10 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="R3" t="n">
-        <v>209792</v>
+        <v>209807</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
@@ -5578,7 +5650,7 @@
         <v>1</v>
       </c>
       <c r="W3" t="n">
-        <v>652794.8476254502</v>
+        <v>652748.5472934669</v>
       </c>
       <c r="X3" t="n">
         <v>14400</v>
@@ -5591,7 +5663,7 @@
         <v>5</v>
       </c>
       <c r="AB3" t="n">
-        <v>157361705.7888646</v>
+        <v>378145902.4795384</v>
       </c>
     </row>
   </sheetData>
@@ -5847,31 +5919,35 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5091186253411937</v>
+        <v>705390119754817</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>6866650600.375151</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+        <v>1220737884.511138</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
         <v>0.75</v>
       </c>
       <c r="L3" t="n">
-        <v>1.15</v>
+        <v>1.05</v>
       </c>
       <c r="M3" t="n">
         <v>20</v>
       </c>
       <c r="N3" t="n">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="O3" t="n">
         <v>0.9</v>
@@ -5882,36 +5958,36 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="R3" t="n">
-        <v>150945</v>
+        <v>51271</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
-        <v>1.5e+20</v>
+        <v>2e+20</v>
       </c>
       <c r="U3" t="n">
-        <v>2.777777777777778e-08</v>
+        <v>6.944444444444444e-08</v>
       </c>
       <c r="V3" t="b">
         <v>1</v>
       </c>
       <c r="W3" t="n">
-        <v>4360994.697124124</v>
+        <v>4315890.926647455</v>
       </c>
       <c r="X3" t="n">
+        <v>21600</v>
+      </c>
+      <c r="Y3" t="n">
         <v>43200</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>7200</v>
       </c>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="n">
         <v>5</v>
       </c>
       <c r="AB3" t="n">
-        <v>141421840.3725538</v>
+        <v>48985424.9829734</v>
       </c>
     </row>
   </sheetData>
@@ -6169,22 +6245,26 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1020416278073986</v>
+        <v>3144972497151465</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>747701954.2630719</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+        <v>6103689422.55569</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
         <v>1.05</v>
@@ -6196,7 +6276,7 @@
         <v>500</v>
       </c>
       <c r="O3" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -6204,36 +6284,36 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="R3" t="n">
-        <v>91925</v>
+        <v>102384</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
-        <v>7e+19</v>
+        <v>2e+20</v>
       </c>
       <c r="U3" t="n">
-        <v>1.111111111111111e-07</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="V3" t="b">
         <v>1</v>
       </c>
       <c r="W3" t="n">
-        <v>8289794.985555269</v>
+        <v>8165327.087865899</v>
       </c>
       <c r="X3" t="n">
-        <v>21600</v>
+        <v>14400</v>
       </c>
       <c r="Y3" t="n">
         <v>7200</v>
       </c>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AB3" t="n">
-        <v>113379586.4526651</v>
+        <v>87360347.14309625</v>
       </c>
     </row>
   </sheetData>
@@ -6489,31 +6569,35 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5165519965489169</v>
+        <v>272270365750398</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>2172581493.312933</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+        <v>94627993.93096329</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
         <v>0.5</v>
       </c>
       <c r="L3" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
       <c r="M3" t="n">
         <v>15</v>
       </c>
       <c r="N3" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="O3" t="n">
         <v>0.9</v>
@@ -6527,11 +6611,11 @@
         <v>0.4</v>
       </c>
       <c r="R3" t="n">
-        <v>80333</v>
+        <v>22499</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
-        <v>1.5e+20</v>
+        <v>7e+19</v>
       </c>
       <c r="U3" t="n">
         <v>1.111111111111111e-07</v>
@@ -6540,7 +6624,7 @@
         <v>1</v>
       </c>
       <c r="W3" t="n">
-        <v>13989385.84561866</v>
+        <v>13768415.33543325</v>
       </c>
       <c r="X3" t="n">
         <v>43200</v>
@@ -6553,7 +6637,7 @@
         <v>5</v>
       </c>
       <c r="AB3" t="n">
-        <v>573946662.8321298</v>
+        <v>30252262.86115533</v>
       </c>
     </row>
   </sheetData>
@@ -6811,35 +6895,35 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ddstartup_20251111_220719_parametric_T_seeded</t>
+          <t>ddstartup_20251112_105650_parametric_T_seeded</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3761915752841065</v>
+        <v>735678291552867.6</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1601740505.970906</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="n">
-        <v>1.262886935408163</v>
-      </c>
-      <c r="J3" t="n">
-        <v>2.361895677493635</v>
-      </c>
+        <v>320348101.1941811</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="L3" t="n">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="M3" t="n">
         <v>10</v>
       </c>
       <c r="N3" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="O3" t="n">
         <v>0.7</v>
@@ -6853,33 +6937,33 @@
         <v>0.3</v>
       </c>
       <c r="R3" t="n">
-        <v>66766</v>
+        <v>16167</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
         <v>2e+20</v>
       </c>
       <c r="U3" t="n">
-        <v>6.944444444444444e-08</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="V3" t="b">
         <v>1</v>
       </c>
       <c r="W3" t="n">
-        <v>24035722.23546692</v>
+        <v>23468644.95781989</v>
       </c>
       <c r="X3" t="n">
-        <v>14400</v>
+        <v>43200</v>
       </c>
       <c r="Y3" t="n">
         <v>43200</v>
       </c>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="AB3" t="n">
-        <v>261244149.5028517</v>
+        <v>20435508.09869077</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new plots for the paper
</commit_message>
<xml_diff>
--- a/outputs/compare_tseeded_lump_t_startup.xlsx
+++ b/outputs/compare_tseeded_lump_t_startup.xlsx
@@ -1535,7 +1535,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.833048159814862e+16</v>
+        <v>1.556198169016034e+16</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
@@ -1566,17 +1566,17 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="P2" t="n">
-        <v>5258038</v>
+        <v>5258005</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
         <v>1.5e+20</v>
       </c>
       <c r="S2" t="n">
-        <v>5.555555555555555e-08</v>
+        <v>8.333333333333333e-08</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -1595,7 +1595,7 @@
         <v>3</v>
       </c>
       <c r="Z2" t="n">
-        <v>1018360088.786034</v>
+        <v>1296831807.513361</v>
       </c>
       <c r="AA2" t="n">
         <v>100</v>
@@ -1776,7 +1776,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.108479023748092e+16</v>
+        <v>1.425187316247547e+16</v>
       </c>
       <c r="E3" t="n">
         <v>1.5</v>
@@ -1801,7 +1801,7 @@
         <v>100</v>
       </c>
       <c r="M3" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
         <v>0.3</v>
       </c>
       <c r="P3" t="n">
-        <v>626867</v>
+        <v>626879</v>
       </c>
       <c r="Q3" t="n">
         <v>2.778955806943149e+16</v>
@@ -1821,7 +1821,7 @@
         <v>2e+20</v>
       </c>
       <c r="S3" t="n">
-        <v>6.944444444444444e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="T3" t="b">
         <v>1</v>
@@ -1838,7 +1838,7 @@
         <v>2.5</v>
       </c>
       <c r="Z3" t="n">
-        <v>769777099.8250638</v>
+        <v>593828048.4364779</v>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
@@ -2402,7 +2402,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>919198771040461.8</v>
+        <v>1193624245971989</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
@@ -2427,7 +2427,7 @@
         <v>100</v>
       </c>
       <c r="M2" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -2435,17 +2435,17 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="P2" t="n">
-        <v>872145</v>
+        <v>872186</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
         <v>7e+19</v>
       </c>
       <c r="S2" t="n">
-        <v>4.166666666666666e-08</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -2464,7 +2464,7 @@
         <v>2</v>
       </c>
       <c r="Z2" t="n">
-        <v>38299948.79335257</v>
+        <v>33156229.05477747</v>
       </c>
       <c r="AA2" t="n">
         <v>100</v>
@@ -2645,7 +2645,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2.598518426070654e+16</v>
+        <v>2.773996327387442e+16</v>
       </c>
       <c r="E3" t="n">
         <v>1.5</v>
@@ -2672,7 +2672,7 @@
         <v>1500</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -2680,10 +2680,10 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="P3" t="n">
-        <v>3067083</v>
+        <v>3067111</v>
       </c>
       <c r="Q3" t="n">
         <v>1416250776663308</v>
@@ -2709,7 +2709,7 @@
         <v>4.5</v>
       </c>
       <c r="Z3" t="n">
-        <v>2526337358.679802</v>
+        <v>2696940873.848902</v>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.138950879990764e+16</v>
+        <v>8542131599930730</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
@@ -3296,7 +3296,7 @@
         <v>1000</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -3307,14 +3307,14 @@
         <v>0.3</v>
       </c>
       <c r="P2" t="n">
-        <v>2666882</v>
+        <v>2666873</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
         <v>1e+20</v>
       </c>
       <c r="S2" t="n">
-        <v>4.166666666666666e-08</v>
+        <v>1.111111111111111e-07</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -3333,7 +3333,7 @@
         <v>3.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>474562866.6628183</v>
+        <v>949125733.3256366</v>
       </c>
       <c r="AA2" t="n">
         <v>100</v>
@@ -3514,16 +3514,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4.645451246323957e+16</v>
+        <v>3.223397464468246e+16</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>392426423.9628718</v>
+        <v>588639635.9443078</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01277628319729316</v>
+        <v>0.01277628319729317</v>
       </c>
       <c r="H3" t="n">
         <v>6.018445976850654</v>
@@ -3538,10 +3538,10 @@
         <v>10</v>
       </c>
       <c r="L3" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -3549,10 +3549,10 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="P3" t="n">
-        <v>2033989</v>
+        <v>3031982</v>
       </c>
       <c r="Q3" t="n">
         <v>1416250776663308</v>
@@ -3561,7 +3561,7 @@
         <v>7e+19</v>
       </c>
       <c r="S3" t="n">
-        <v>1.111111111111111e-07</v>
+        <v>5.555555555555555e-08</v>
       </c>
       <c r="T3" t="b">
         <v>1</v>
@@ -3578,7 +3578,7 @@
         <v>2.5</v>
       </c>
       <c r="Z3" t="n">
-        <v>5161612495.915507</v>
+        <v>1790776369.149026</v>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
@@ -3596,79 +3596,79 @@
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AQ3" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AR3" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AS3" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AT3" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AU3" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AV3" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AW3" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AX3" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AY3" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AZ3" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BA3" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BB3" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BC3" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BD3" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BE3" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BF3" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BG3" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BH3" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BI3" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BJ3" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BK3" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BL3" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BM3" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BN3" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BO3" t="inlineStr"/>
       <c r="BP3" t="inlineStr"/>
@@ -4150,7 +4150,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>806518874978931.2</v>
+        <v>705704015606564.8</v>
       </c>
       <c r="F2" t="n">
         <v>0.1</v>
@@ -4175,7 +4175,7 @@
         <v>2000</v>
       </c>
       <c r="N2" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -4186,7 +4186,7 @@
         <v>0.4</v>
       </c>
       <c r="Q2" t="n">
-        <v>4988820</v>
+        <v>4988812</v>
       </c>
       <c r="R2" t="n">
         <v>4.79379534335385e+16</v>
@@ -4195,7 +4195,7 @@
         <v>2e+20</v>
       </c>
       <c r="T2" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>6.944444444444444e-08</v>
       </c>
       <c r="U2" t="b">
         <v>1</v>
@@ -4212,7 +4212,7 @@
         <v>5</v>
       </c>
       <c r="AA2" t="n">
-        <v>67209906.24824427</v>
+        <v>49007223.30601144</v>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
@@ -4358,7 +4358,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1987191529253553</v>
+        <v>1655992941044627</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
@@ -4381,7 +4381,7 @@
         <v>2000</v>
       </c>
       <c r="N3" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -4392,14 +4392,14 @@
         <v>0.3</v>
       </c>
       <c r="Q3" t="n">
-        <v>6235961</v>
+        <v>6235951</v>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="n">
         <v>2e+20</v>
       </c>
       <c r="T3" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="U3" t="b">
         <v>1</v>
@@ -4418,7 +4418,7 @@
         <v>5</v>
       </c>
       <c r="AA3" t="n">
-        <v>165599294.1044627</v>
+        <v>68999705.87685946</v>
       </c>
       <c r="AB3" t="n">
         <v>100</v>
@@ -4602,7 +4602,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1006157420309785</v>
+        <v>839564548444715.8</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
@@ -4633,17 +4633,17 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>3010415</v>
+        <v>3010383</v>
       </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="n">
         <v>7e+19</v>
       </c>
       <c r="T4" t="n">
-        <v>5.555555555555555e-08</v>
+        <v>9.722222222222221e-08</v>
       </c>
       <c r="U4" t="b">
         <v>1</v>
@@ -4662,7 +4662,7 @@
         <v>5</v>
       </c>
       <c r="AA4" t="n">
-        <v>55897634.46165472</v>
+        <v>81624331.09879179</v>
       </c>
       <c r="AB4" t="n">
         <v>100</v>
@@ -4846,13 +4846,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1.288108944550896e+16</v>
+        <v>2.00372502485695e+16</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>7724734198.445983</v>
+        <v>15449468396.89197</v>
       </c>
       <c r="H5" t="n">
         <v>0.08449193122405596</v>
@@ -4868,10 +4868,10 @@
         <v>15</v>
       </c>
       <c r="M5" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="N5" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -4882,7 +4882,7 @@
         <v>0.4</v>
       </c>
       <c r="Q5" t="n">
-        <v>2624367</v>
+        <v>4620329</v>
       </c>
       <c r="R5" t="n">
         <v>2.778955806943149e+16</v>
@@ -4891,7 +4891,7 @@
         <v>2e+20</v>
       </c>
       <c r="T5" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="U5" t="b">
         <v>1</v>
@@ -4908,7 +4908,7 @@
         <v>3</v>
       </c>
       <c r="AA5" t="n">
-        <v>1073424120.45908</v>
+        <v>556590284.6824861</v>
       </c>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
@@ -4926,64 +4926,64 @@
       <c r="AO5" t="inlineStr"/>
       <c r="AP5" t="inlineStr"/>
       <c r="AQ5" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AR5" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AS5" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AT5" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AU5" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AV5" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AW5" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AX5" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AY5" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AZ5" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="BA5" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BB5" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BC5" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BD5" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BE5" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BF5" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BG5" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BH5" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BI5" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BJ5" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BK5" t="n">
         <v>0</v>
@@ -5054,7 +5054,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4940562124033113</v>
+        <v>3945663403034427</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
@@ -5077,7 +5077,7 @@
         <v>1000</v>
       </c>
       <c r="N6" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -5085,17 +5085,17 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="Q6" t="n">
-        <v>2862614</v>
+        <v>2862624</v>
       </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="n">
         <v>2e+20</v>
       </c>
       <c r="T6" t="n">
-        <v>1.111111111111111e-07</v>
+        <v>5.555555555555555e-08</v>
       </c>
       <c r="U6" t="b">
         <v>1</v>
@@ -5114,7 +5114,7 @@
         <v>2.5</v>
       </c>
       <c r="AA6" t="n">
-        <v>548951347.1147903</v>
+        <v>219203522.3908015</v>
       </c>
       <c r="AB6" t="n">
         <v>100</v>
@@ -5298,7 +5298,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1.759712215371368e+16</v>
+        <v>2.463597101519915e+16</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
@@ -5323,7 +5323,7 @@
         <v>1000</v>
       </c>
       <c r="N7" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -5334,14 +5334,14 @@
         <v>0.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>3651970</v>
+        <v>3651985</v>
       </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="n">
         <v>2e+20</v>
       </c>
       <c r="T7" t="n">
-        <v>2.777777777777778e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="U7" t="b">
         <v>1</v>
@@ -5360,7 +5360,7 @@
         <v>0.5</v>
       </c>
       <c r="AA7" t="n">
-        <v>488808948.7142688</v>
+        <v>1026498792.299964</v>
       </c>
       <c r="AB7" t="n">
         <v>100</v>
@@ -5544,19 +5544,19 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3.813384400652378e+16</v>
+        <v>1.145001421325982e+16</v>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>10299975900.56273</v>
+        <v>3433325300.187575</v>
       </c>
       <c r="H8" t="n">
         <v>0.01248575833914265</v>
       </c>
       <c r="I8" t="n">
-        <v>4.359222671561555</v>
+        <v>4.359222671561554</v>
       </c>
       <c r="J8" t="n">
         <v>0.5</v>
@@ -5568,10 +5568,10 @@
         <v>20</v>
       </c>
       <c r="M8" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="N8" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -5579,10 +5579,10 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="Q8" t="n">
-        <v>3838402</v>
+        <v>1842303</v>
       </c>
       <c r="R8" t="n">
         <v>2.696979113134065e+16</v>
@@ -5608,7 +5608,7 @@
         <v>0.5</v>
       </c>
       <c r="AA8" t="n">
-        <v>1588910166.938491</v>
+        <v>477083925.5524923</v>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
@@ -5626,79 +5626,79 @@
       <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AR8" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AS8" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AT8" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AU8" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AV8" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AW8" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AX8" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AY8" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AZ8" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="BA8" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BB8" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BC8" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BD8" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BE8" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BF8" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BG8" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BH8" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BI8" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BJ8" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BK8" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BL8" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BM8" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BN8" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BO8" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BP8" t="inlineStr"/>
       <c r="BQ8" t="inlineStr"/>
@@ -5754,7 +5754,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3.113260860270707e+16</v>
+        <v>2.671953057464017e+16</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
@@ -5787,17 +5787,17 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="Q9" t="n">
-        <v>3238540</v>
+        <v>3238507</v>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
         <v>2e+20</v>
       </c>
       <c r="T9" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>1.111111111111111e-07</v>
       </c>
       <c r="U9" t="b">
         <v>1</v>
@@ -5816,7 +5816,7 @@
         <v>0.5</v>
       </c>
       <c r="AA9" t="n">
-        <v>2594384050.225589</v>
+        <v>2968836730.515574</v>
       </c>
       <c r="AB9" t="n">
         <v>100</v>
@@ -6000,7 +6000,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1.833048159814862e+16</v>
+        <v>1.556198169016034e+16</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
@@ -6031,17 +6031,17 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>5258038</v>
+        <v>5258005</v>
       </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
         <v>1.5e+20</v>
       </c>
       <c r="T10" t="n">
-        <v>5.555555555555555e-08</v>
+        <v>8.333333333333333e-08</v>
       </c>
       <c r="U10" t="b">
         <v>1</v>
@@ -6060,7 +6060,7 @@
         <v>3</v>
       </c>
       <c r="AA10" t="n">
-        <v>1018360088.786034</v>
+        <v>1296831807.513361</v>
       </c>
       <c r="AB10" t="n">
         <v>100</v>
@@ -6244,13 +6244,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2.794826622829694e+16</v>
+        <v>1.676895973697816e+16</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>6866650600.375151</v>
+        <v>3433325300.187575</v>
       </c>
       <c r="H11" t="n">
         <v>0.1472880275120053</v>
@@ -6266,10 +6266,10 @@
         <v>20</v>
       </c>
       <c r="M11" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="N11" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -6280,7 +6280,7 @@
         <v>0.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>2901117</v>
+        <v>1902924</v>
       </c>
       <c r="R11" t="n">
         <v>2.696979113134065e+16</v>
@@ -6306,7 +6306,7 @@
         <v>4.5</v>
       </c>
       <c r="AA11" t="n">
-        <v>1552681457.127608</v>
+        <v>931608874.2765646</v>
       </c>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
@@ -6324,64 +6324,64 @@
       <c r="AO11" t="inlineStr"/>
       <c r="AP11" t="inlineStr"/>
       <c r="AQ11" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AR11" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AS11" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AT11" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AU11" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AV11" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AW11" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AX11" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AY11" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AZ11" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="BA11" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BB11" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BC11" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BD11" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BE11" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BF11" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BG11" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BH11" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BI11" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BJ11" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BK11" t="n">
         <v>0</v>
@@ -6452,7 +6452,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>919198771040461.8</v>
+        <v>1193624245971989</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
@@ -6477,7 +6477,7 @@
         <v>100</v>
       </c>
       <c r="N12" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -6485,17 +6485,17 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="Q12" t="n">
-        <v>872145</v>
+        <v>872186</v>
       </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="n">
         <v>7e+19</v>
       </c>
       <c r="T12" t="n">
-        <v>4.166666666666666e-08</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="U12" t="b">
         <v>1</v>
@@ -6514,7 +6514,7 @@
         <v>2</v>
       </c>
       <c r="AA12" t="n">
-        <v>38299948.79335257</v>
+        <v>33156229.05477747</v>
       </c>
       <c r="AB12" t="n">
         <v>100</v>
@@ -6698,13 +6698,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3917755605130725</v>
+        <v>1.175326681539218e+17</v>
       </c>
       <c r="F13" t="n">
-        <v>0.5</v>
+        <v>10</v>
       </c>
       <c r="G13" t="n">
-        <v>434516298.6625866</v>
+        <v>8690325973.251732</v>
       </c>
       <c r="H13" t="n">
         <v>0.0291640551121764</v>
@@ -6720,10 +6720,10 @@
         <v>15</v>
       </c>
       <c r="M13" t="n">
-        <v>100</v>
+        <v>2000</v>
       </c>
       <c r="N13" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -6734,7 +6734,7 @@
         <v>0.3</v>
       </c>
       <c r="Q13" t="n">
-        <v>523399</v>
+        <v>4515799</v>
       </c>
       <c r="R13" t="n">
         <v>1.563254491497592e+16</v>
@@ -6743,7 +6743,7 @@
         <v>1.5e+20</v>
       </c>
       <c r="T13" t="n">
-        <v>5.555555555555555e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="U13" t="b">
         <v>1</v>
@@ -6760,7 +6760,7 @@
         <v>1.5</v>
       </c>
       <c r="AA13" t="n">
-        <v>217653089.1739292</v>
+        <v>4897194506.413406</v>
       </c>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
@@ -6778,64 +6778,64 @@
       <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AR13" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AS13" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AT13" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AU13" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AV13" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AW13" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AX13" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AY13" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AZ13" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="BA13" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BB13" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BC13" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BD13" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BE13" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BF13" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BG13" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BH13" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BI13" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BJ13" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BK13" t="n">
         <v>0</v>
@@ -6906,7 +6906,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1.108479023748092e+16</v>
+        <v>1.425187316247547e+16</v>
       </c>
       <c r="F14" t="n">
         <v>1.5</v>
@@ -6931,7 +6931,7 @@
         <v>100</v>
       </c>
       <c r="N14" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -6942,7 +6942,7 @@
         <v>0.3</v>
       </c>
       <c r="Q14" t="n">
-        <v>626867</v>
+        <v>626879</v>
       </c>
       <c r="R14" t="n">
         <v>2.778955806943149e+16</v>
@@ -6951,7 +6951,7 @@
         <v>2e+20</v>
       </c>
       <c r="T14" t="n">
-        <v>6.944444444444444e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="U14" t="b">
         <v>1</v>
@@ -6968,7 +6968,7 @@
         <v>2.5</v>
       </c>
       <c r="AA14" t="n">
-        <v>769777099.8250638</v>
+        <v>593828048.4364779</v>
       </c>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
@@ -7114,7 +7114,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1.138950879990764e+16</v>
+        <v>8542131599930730</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
@@ -7137,7 +7137,7 @@
         <v>1000</v>
       </c>
       <c r="N15" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -7148,14 +7148,14 @@
         <v>0.3</v>
       </c>
       <c r="Q15" t="n">
-        <v>2666882</v>
+        <v>2666873</v>
       </c>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="n">
         <v>1e+20</v>
       </c>
       <c r="T15" t="n">
-        <v>4.166666666666666e-08</v>
+        <v>1.111111111111111e-07</v>
       </c>
       <c r="U15" t="b">
         <v>1</v>
@@ -7174,7 +7174,7 @@
         <v>3.5</v>
       </c>
       <c r="AA15" t="n">
-        <v>474562866.6628183</v>
+        <v>949125733.3256366</v>
       </c>
       <c r="AB15" t="n">
         <v>100</v>
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>2.598518426070654e+16</v>
+        <v>2.773996327387442e+16</v>
       </c>
       <c r="F16" t="n">
         <v>1.5</v>
@@ -7385,7 +7385,7 @@
         <v>1500</v>
       </c>
       <c r="N16" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -7393,10 +7393,10 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>3067083</v>
+        <v>3067111</v>
       </c>
       <c r="R16" t="n">
         <v>1416250776663308</v>
@@ -7422,7 +7422,7 @@
         <v>4.5</v>
       </c>
       <c r="AA16" t="n">
-        <v>2526337358.679802</v>
+        <v>2696940873.848902</v>
       </c>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
@@ -7568,16 +7568,16 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>4.645451246323957e+16</v>
+        <v>3.223397464468246e+16</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17" t="n">
-        <v>392426423.9628718</v>
+        <v>588639635.9443078</v>
       </c>
       <c r="H17" t="n">
-        <v>0.01277628319729316</v>
+        <v>0.01277628319729317</v>
       </c>
       <c r="I17" t="n">
         <v>6.018445976850654</v>
@@ -7592,10 +7592,10 @@
         <v>10</v>
       </c>
       <c r="M17" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="N17" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -7603,10 +7603,10 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="Q17" t="n">
-        <v>2033989</v>
+        <v>3031982</v>
       </c>
       <c r="R17" t="n">
         <v>1416250776663308</v>
@@ -7615,7 +7615,7 @@
         <v>7e+19</v>
       </c>
       <c r="T17" t="n">
-        <v>1.111111111111111e-07</v>
+        <v>5.555555555555555e-08</v>
       </c>
       <c r="U17" t="b">
         <v>1</v>
@@ -7632,7 +7632,7 @@
         <v>2.5</v>
       </c>
       <c r="AA17" t="n">
-        <v>5161612495.915507</v>
+        <v>1790776369.149026</v>
       </c>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
@@ -7650,79 +7650,79 @@
       <c r="AO17" t="inlineStr"/>
       <c r="AP17" t="inlineStr"/>
       <c r="AQ17" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AR17" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AS17" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AT17" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AU17" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AV17" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AW17" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AX17" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AY17" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AZ17" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="BA17" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BB17" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BC17" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BD17" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BE17" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BF17" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BG17" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BH17" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BI17" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BJ17" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BK17" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BL17" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BM17" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BN17" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BO17" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BP17" t="inlineStr"/>
       <c r="BQ17" t="inlineStr"/>
@@ -8196,7 +8196,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1987191529253553</v>
+        <v>1655992941044627</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
@@ -8219,7 +8219,7 @@
         <v>2000</v>
       </c>
       <c r="M2" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -8230,14 +8230,14 @@
         <v>0.3</v>
       </c>
       <c r="P2" t="n">
-        <v>6235961</v>
+        <v>6235951</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
         <v>2e+20</v>
       </c>
       <c r="S2" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -8256,7 +8256,7 @@
         <v>5</v>
       </c>
       <c r="Z2" t="n">
-        <v>165599294.1044627</v>
+        <v>68999705.87685946</v>
       </c>
       <c r="AA2" t="n">
         <v>100</v>
@@ -8437,7 +8437,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1006157420309785</v>
+        <v>839564548444715.8</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
@@ -8468,17 +8468,17 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="P3" t="n">
-        <v>3010415</v>
+        <v>3010383</v>
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="n">
         <v>7e+19</v>
       </c>
       <c r="S3" t="n">
-        <v>5.555555555555555e-08</v>
+        <v>9.722222222222221e-08</v>
       </c>
       <c r="T3" t="b">
         <v>1</v>
@@ -8497,7 +8497,7 @@
         <v>5</v>
       </c>
       <c r="Z3" t="n">
-        <v>55897634.46165472</v>
+        <v>81624331.09879179</v>
       </c>
       <c r="AA3" t="n">
         <v>100</v>
@@ -8678,7 +8678,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4940562124033113</v>
+        <v>3945663403034427</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
@@ -8701,7 +8701,7 @@
         <v>1000</v>
       </c>
       <c r="M4" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -8709,17 +8709,17 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="P4" t="n">
-        <v>2862614</v>
+        <v>2862624</v>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="n">
         <v>2e+20</v>
       </c>
       <c r="S4" t="n">
-        <v>1.111111111111111e-07</v>
+        <v>5.555555555555555e-08</v>
       </c>
       <c r="T4" t="b">
         <v>1</v>
@@ -8738,7 +8738,7 @@
         <v>2.5</v>
       </c>
       <c r="Z4" t="n">
-        <v>548951347.1147903</v>
+        <v>219203522.3908015</v>
       </c>
       <c r="AA4" t="n">
         <v>100</v>
@@ -8919,7 +8919,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.759712215371368e+16</v>
+        <v>2.463597101519915e+16</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
@@ -8944,7 +8944,7 @@
         <v>1000</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -8955,14 +8955,14 @@
         <v>0.3</v>
       </c>
       <c r="P5" t="n">
-        <v>3651970</v>
+        <v>3651985</v>
       </c>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="n">
         <v>2e+20</v>
       </c>
       <c r="S5" t="n">
-        <v>2.777777777777778e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="T5" t="b">
         <v>1</v>
@@ -8981,7 +8981,7 @@
         <v>0.5</v>
       </c>
       <c r="Z5" t="n">
-        <v>488808948.7142688</v>
+        <v>1026498792.299964</v>
       </c>
       <c r="AA5" t="n">
         <v>100</v>
@@ -9162,7 +9162,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3.113260860270707e+16</v>
+        <v>2.671953057464017e+16</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
@@ -9195,17 +9195,17 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="P6" t="n">
-        <v>3238540</v>
+        <v>3238507</v>
       </c>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="n">
         <v>2e+20</v>
       </c>
       <c r="S6" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>1.111111111111111e-07</v>
       </c>
       <c r="T6" t="b">
         <v>1</v>
@@ -9224,7 +9224,7 @@
         <v>0.5</v>
       </c>
       <c r="Z6" t="n">
-        <v>2594384050.225589</v>
+        <v>2968836730.515574</v>
       </c>
       <c r="AA6" t="n">
         <v>100</v>
@@ -9405,7 +9405,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.833048159814862e+16</v>
+        <v>1.556198169016034e+16</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
@@ -9436,17 +9436,17 @@
         </is>
       </c>
       <c r="O7" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="P7" t="n">
-        <v>5258038</v>
+        <v>5258005</v>
       </c>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="n">
         <v>1.5e+20</v>
       </c>
       <c r="S7" t="n">
-        <v>5.555555555555555e-08</v>
+        <v>8.333333333333333e-08</v>
       </c>
       <c r="T7" t="b">
         <v>1</v>
@@ -9465,7 +9465,7 @@
         <v>3</v>
       </c>
       <c r="Z7" t="n">
-        <v>1018360088.786034</v>
+        <v>1296831807.513361</v>
       </c>
       <c r="AA7" t="n">
         <v>100</v>
@@ -9646,7 +9646,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>919198771040461.8</v>
+        <v>1193624245971989</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
@@ -9671,7 +9671,7 @@
         <v>100</v>
       </c>
       <c r="M8" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -9679,17 +9679,17 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="P8" t="n">
-        <v>872145</v>
+        <v>872186</v>
       </c>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="n">
         <v>7e+19</v>
       </c>
       <c r="S8" t="n">
-        <v>4.166666666666666e-08</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="T8" t="b">
         <v>1</v>
@@ -9708,7 +9708,7 @@
         <v>2</v>
       </c>
       <c r="Z8" t="n">
-        <v>38299948.79335257</v>
+        <v>33156229.05477747</v>
       </c>
       <c r="AA8" t="n">
         <v>100</v>
@@ -9889,7 +9889,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.138950879990764e+16</v>
+        <v>8542131599930730</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
@@ -9912,7 +9912,7 @@
         <v>1000</v>
       </c>
       <c r="M9" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -9923,14 +9923,14 @@
         <v>0.3</v>
       </c>
       <c r="P9" t="n">
-        <v>2666882</v>
+        <v>2666873</v>
       </c>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="n">
         <v>1e+20</v>
       </c>
       <c r="S9" t="n">
-        <v>4.166666666666666e-08</v>
+        <v>1.111111111111111e-07</v>
       </c>
       <c r="T9" t="b">
         <v>1</v>
@@ -9949,7 +9949,7 @@
         <v>3.5</v>
       </c>
       <c r="Z9" t="n">
-        <v>474562866.6628183</v>
+        <v>949125733.3256366</v>
       </c>
       <c r="AA9" t="n">
         <v>100</v>
@@ -10551,7 +10551,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>806518874978931.2</v>
+        <v>705704015606564.8</v>
       </c>
       <c r="E2" t="n">
         <v>0.1</v>
@@ -10576,7 +10576,7 @@
         <v>2000</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -10587,7 +10587,7 @@
         <v>0.4</v>
       </c>
       <c r="P2" t="n">
-        <v>4988820</v>
+        <v>4988812</v>
       </c>
       <c r="Q2" t="n">
         <v>4.79379534335385e+16</v>
@@ -10596,7 +10596,7 @@
         <v>2e+20</v>
       </c>
       <c r="S2" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>6.944444444444444e-08</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -10613,7 +10613,7 @@
         <v>5</v>
       </c>
       <c r="Z2" t="n">
-        <v>67209906.24824427</v>
+        <v>49007223.30601144</v>
       </c>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
@@ -10756,13 +10756,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.288108944550896e+16</v>
+        <v>2.00372502485695e+16</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>7724734198.445983</v>
+        <v>15449468396.89197</v>
       </c>
       <c r="G3" t="n">
         <v>0.08449193122405596</v>
@@ -10778,10 +10778,10 @@
         <v>15</v>
       </c>
       <c r="L3" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -10792,7 +10792,7 @@
         <v>0.4</v>
       </c>
       <c r="P3" t="n">
-        <v>2624367</v>
+        <v>4620329</v>
       </c>
       <c r="Q3" t="n">
         <v>2.778955806943149e+16</v>
@@ -10801,7 +10801,7 @@
         <v>2e+20</v>
       </c>
       <c r="S3" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="T3" t="b">
         <v>1</v>
@@ -10818,7 +10818,7 @@
         <v>3</v>
       </c>
       <c r="Z3" t="n">
-        <v>1073424120.45908</v>
+        <v>556590284.6824861</v>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
@@ -10836,64 +10836,64 @@
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AQ3" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AR3" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AS3" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AT3" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AU3" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AV3" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AW3" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AX3" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AY3" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AZ3" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BA3" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BB3" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BC3" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BD3" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BE3" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BF3" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BG3" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BH3" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BI3" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BJ3" t="n">
         <v>0</v>
@@ -10961,19 +10961,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.813384400652378e+16</v>
+        <v>1.145001421325982e+16</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>10299975900.56273</v>
+        <v>3433325300.187575</v>
       </c>
       <c r="G4" t="n">
         <v>0.01248575833914265</v>
       </c>
       <c r="H4" t="n">
-        <v>4.359222671561555</v>
+        <v>4.359222671561554</v>
       </c>
       <c r="I4" t="n">
         <v>0.5</v>
@@ -10985,10 +10985,10 @@
         <v>20</v>
       </c>
       <c r="L4" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="M4" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -10996,10 +10996,10 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="P4" t="n">
-        <v>3838402</v>
+        <v>1842303</v>
       </c>
       <c r="Q4" t="n">
         <v>2.696979113134065e+16</v>
@@ -11025,7 +11025,7 @@
         <v>0.5</v>
       </c>
       <c r="Z4" t="n">
-        <v>1588910166.938491</v>
+        <v>477083925.5524923</v>
       </c>
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
@@ -11043,79 +11043,79 @@
       <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="inlineStr"/>
       <c r="AP4" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AQ4" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AR4" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AS4" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AT4" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AU4" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AV4" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AW4" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AX4" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AY4" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AZ4" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BA4" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BB4" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BC4" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BD4" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BE4" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BF4" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BG4" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BH4" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BI4" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BJ4" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BK4" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BL4" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BM4" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BN4" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BO4" t="inlineStr"/>
       <c r="BP4" t="inlineStr"/>
@@ -11168,13 +11168,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2.794826622829694e+16</v>
+        <v>1.676895973697816e+16</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>6866650600.375151</v>
+        <v>3433325300.187575</v>
       </c>
       <c r="G5" t="n">
         <v>0.1472880275120053</v>
@@ -11190,10 +11190,10 @@
         <v>20</v>
       </c>
       <c r="L5" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -11204,7 +11204,7 @@
         <v>0.4</v>
       </c>
       <c r="P5" t="n">
-        <v>2901117</v>
+        <v>1902924</v>
       </c>
       <c r="Q5" t="n">
         <v>2.696979113134065e+16</v>
@@ -11230,7 +11230,7 @@
         <v>4.5</v>
       </c>
       <c r="Z5" t="n">
-        <v>1552681457.127608</v>
+        <v>931608874.2765646</v>
       </c>
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
@@ -11248,64 +11248,64 @@
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
       <c r="AP5" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AQ5" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AR5" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AS5" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AT5" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AU5" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AV5" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AW5" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AX5" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AY5" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AZ5" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BA5" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BB5" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BC5" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BD5" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BE5" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BF5" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BG5" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BH5" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BI5" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BJ5" t="n">
         <v>0</v>
@@ -11373,13 +11373,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3917755605130725</v>
+        <v>1.175326681539218e+17</v>
       </c>
       <c r="E6" t="n">
-        <v>0.5</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>434516298.6625866</v>
+        <v>8690325973.251732</v>
       </c>
       <c r="G6" t="n">
         <v>0.0291640551121764</v>
@@ -11395,10 +11395,10 @@
         <v>15</v>
       </c>
       <c r="L6" t="n">
-        <v>100</v>
+        <v>2000</v>
       </c>
       <c r="M6" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -11409,7 +11409,7 @@
         <v>0.3</v>
       </c>
       <c r="P6" t="n">
-        <v>523399</v>
+        <v>4515799</v>
       </c>
       <c r="Q6" t="n">
         <v>1.563254491497592e+16</v>
@@ -11418,7 +11418,7 @@
         <v>1.5e+20</v>
       </c>
       <c r="S6" t="n">
-        <v>5.555555555555555e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="T6" t="b">
         <v>1</v>
@@ -11435,7 +11435,7 @@
         <v>1.5</v>
       </c>
       <c r="Z6" t="n">
-        <v>217653089.1739292</v>
+        <v>4897194506.413406</v>
       </c>
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
@@ -11453,64 +11453,64 @@
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
       <c r="AP6" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AQ6" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AR6" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AS6" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AT6" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AU6" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AV6" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AW6" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AX6" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AY6" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AZ6" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BA6" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BB6" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BC6" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BD6" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BE6" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BF6" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BG6" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BH6" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BI6" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BJ6" t="n">
         <v>0</v>
@@ -11578,7 +11578,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.108479023748092e+16</v>
+        <v>1.425187316247547e+16</v>
       </c>
       <c r="E7" t="n">
         <v>1.5</v>
@@ -11603,7 +11603,7 @@
         <v>100</v>
       </c>
       <c r="M7" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -11614,7 +11614,7 @@
         <v>0.3</v>
       </c>
       <c r="P7" t="n">
-        <v>626867</v>
+        <v>626879</v>
       </c>
       <c r="Q7" t="n">
         <v>2.778955806943149e+16</v>
@@ -11623,7 +11623,7 @@
         <v>2e+20</v>
       </c>
       <c r="S7" t="n">
-        <v>6.944444444444444e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="T7" t="b">
         <v>1</v>
@@ -11640,7 +11640,7 @@
         <v>2.5</v>
       </c>
       <c r="Z7" t="n">
-        <v>769777099.8250638</v>
+        <v>593828048.4364779</v>
       </c>
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
@@ -11783,7 +11783,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2.598518426070654e+16</v>
+        <v>2.773996327387442e+16</v>
       </c>
       <c r="E8" t="n">
         <v>1.5</v>
@@ -11810,7 +11810,7 @@
         <v>1500</v>
       </c>
       <c r="M8" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -11818,10 +11818,10 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="P8" t="n">
-        <v>3067083</v>
+        <v>3067111</v>
       </c>
       <c r="Q8" t="n">
         <v>1416250776663308</v>
@@ -11847,7 +11847,7 @@
         <v>4.5</v>
       </c>
       <c r="Z8" t="n">
-        <v>2526337358.679802</v>
+        <v>2696940873.848902</v>
       </c>
       <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
@@ -11990,16 +11990,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>4.645451246323957e+16</v>
+        <v>3.223397464468246e+16</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>392426423.9628718</v>
+        <v>588639635.9443078</v>
       </c>
       <c r="G9" t="n">
-        <v>0.01277628319729316</v>
+        <v>0.01277628319729317</v>
       </c>
       <c r="H9" t="n">
         <v>6.018445976850654</v>
@@ -12014,10 +12014,10 @@
         <v>10</v>
       </c>
       <c r="L9" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="M9" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -12025,10 +12025,10 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="P9" t="n">
-        <v>2033989</v>
+        <v>3031982</v>
       </c>
       <c r="Q9" t="n">
         <v>1416250776663308</v>
@@ -12037,7 +12037,7 @@
         <v>7e+19</v>
       </c>
       <c r="S9" t="n">
-        <v>1.111111111111111e-07</v>
+        <v>5.555555555555555e-08</v>
       </c>
       <c r="T9" t="b">
         <v>1</v>
@@ -12054,7 +12054,7 @@
         <v>2.5</v>
       </c>
       <c r="Z9" t="n">
-        <v>5161612495.915507</v>
+        <v>1790776369.149026</v>
       </c>
       <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
@@ -12072,79 +12072,79 @@
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AQ9" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AR9" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AS9" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AT9" t="n">
-        <v>785114.7144859461</v>
+        <v>1177672.071728919</v>
       </c>
       <c r="AU9" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AV9" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AW9" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AX9" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AY9" t="n">
-        <v>952809.9117682836</v>
+        <v>1429214.867652426</v>
       </c>
       <c r="AZ9" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BA9" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BB9" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BC9" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BD9" t="n">
-        <v>81115.07036891115</v>
+        <v>121672.6055533667</v>
       </c>
       <c r="BE9" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BF9" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BG9" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BH9" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BI9" t="n">
-        <v>142381043.5012</v>
+        <v>213571565.2517999</v>
       </c>
       <c r="BJ9" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BK9" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BL9" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BM9" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BN9" t="n">
-        <v>65203945.58201578</v>
+        <v>97805918.37302366</v>
       </c>
       <c r="BO9" t="inlineStr"/>
       <c r="BP9" t="inlineStr"/>
@@ -12618,7 +12618,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>806518874978931.2</v>
+        <v>705704015606564.8</v>
       </c>
       <c r="E2" t="n">
         <v>0.1</v>
@@ -12643,7 +12643,7 @@
         <v>2000</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -12654,7 +12654,7 @@
         <v>0.4</v>
       </c>
       <c r="P2" t="n">
-        <v>4988820</v>
+        <v>4988812</v>
       </c>
       <c r="Q2" t="n">
         <v>4.79379534335385e+16</v>
@@ -12663,7 +12663,7 @@
         <v>2e+20</v>
       </c>
       <c r="S2" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>6.944444444444444e-08</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -12680,7 +12680,7 @@
         <v>5</v>
       </c>
       <c r="Z2" t="n">
-        <v>67209906.24824427</v>
+        <v>49007223.30601144</v>
       </c>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
@@ -12823,7 +12823,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1987191529253553</v>
+        <v>1655992941044627</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
@@ -12846,7 +12846,7 @@
         <v>2000</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -12857,14 +12857,14 @@
         <v>0.3</v>
       </c>
       <c r="P3" t="n">
-        <v>6235961</v>
+        <v>6235951</v>
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="n">
         <v>2e+20</v>
       </c>
       <c r="S3" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="T3" t="b">
         <v>1</v>
@@ -12883,7 +12883,7 @@
         <v>5</v>
       </c>
       <c r="Z3" t="n">
-        <v>165599294.1044627</v>
+        <v>68999705.87685946</v>
       </c>
       <c r="AA3" t="n">
         <v>100</v>
@@ -13485,7 +13485,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1006157420309785</v>
+        <v>839564548444715.8</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
@@ -13516,17 +13516,17 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="P2" t="n">
-        <v>3010415</v>
+        <v>3010383</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
         <v>7e+19</v>
       </c>
       <c r="S2" t="n">
-        <v>5.555555555555555e-08</v>
+        <v>9.722222222222221e-08</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -13545,7 +13545,7 @@
         <v>5</v>
       </c>
       <c r="Z2" t="n">
-        <v>55897634.46165472</v>
+        <v>81624331.09879179</v>
       </c>
       <c r="AA2" t="n">
         <v>100</v>
@@ -13726,13 +13726,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.288108944550896e+16</v>
+        <v>2.00372502485695e+16</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>7724734198.445983</v>
+        <v>15449468396.89197</v>
       </c>
       <c r="G3" t="n">
         <v>0.08449193122405596</v>
@@ -13748,10 +13748,10 @@
         <v>15</v>
       </c>
       <c r="L3" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -13762,7 +13762,7 @@
         <v>0.4</v>
       </c>
       <c r="P3" t="n">
-        <v>2624367</v>
+        <v>4620329</v>
       </c>
       <c r="Q3" t="n">
         <v>2.778955806943149e+16</v>
@@ -13771,7 +13771,7 @@
         <v>2e+20</v>
       </c>
       <c r="S3" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>2.777777777777778e-08</v>
       </c>
       <c r="T3" t="b">
         <v>1</v>
@@ -13788,7 +13788,7 @@
         <v>3</v>
       </c>
       <c r="Z3" t="n">
-        <v>1073424120.45908</v>
+        <v>556590284.6824861</v>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
@@ -13806,64 +13806,64 @@
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AQ3" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AR3" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AS3" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AT3" t="n">
-        <v>15408849.52055439</v>
+        <v>30817699.04110878</v>
       </c>
       <c r="AU3" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AV3" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AW3" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AX3" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AY3" t="n">
-        <v>19127301.86048525</v>
+        <v>38254603.7209705</v>
       </c>
       <c r="AZ3" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BA3" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BB3" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BC3" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BD3" t="n">
-        <v>11791894.56292444</v>
+        <v>23583789.12584888</v>
       </c>
       <c r="BE3" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BF3" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BG3" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BH3" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BI3" t="n">
-        <v>548536423.4966457</v>
+        <v>1097072846.993291</v>
       </c>
       <c r="BJ3" t="n">
         <v>0</v>
@@ -14352,7 +14352,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4940562124033113</v>
+        <v>3945663403034427</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
@@ -14375,7 +14375,7 @@
         <v>1000</v>
       </c>
       <c r="M2" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -14383,17 +14383,17 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="P2" t="n">
-        <v>2862614</v>
+        <v>2862624</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
         <v>2e+20</v>
       </c>
       <c r="S2" t="n">
-        <v>1.111111111111111e-07</v>
+        <v>5.555555555555555e-08</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -14412,7 +14412,7 @@
         <v>2.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>548951347.1147903</v>
+        <v>219203522.3908015</v>
       </c>
       <c r="AA2" t="n">
         <v>100</v>
@@ -14593,19 +14593,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3.813384400652378e+16</v>
+        <v>1.145001421325982e+16</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>10299975900.56273</v>
+        <v>3433325300.187575</v>
       </c>
       <c r="G3" t="n">
         <v>0.01248575833914265</v>
       </c>
       <c r="H3" t="n">
-        <v>4.359222671561555</v>
+        <v>4.359222671561554</v>
       </c>
       <c r="I3" t="n">
         <v>0.5</v>
@@ -14617,10 +14617,10 @@
         <v>20</v>
       </c>
       <c r="L3" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -14628,10 +14628,10 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="P3" t="n">
-        <v>3838402</v>
+        <v>1842303</v>
       </c>
       <c r="Q3" t="n">
         <v>2.696979113134065e+16</v>
@@ -14657,7 +14657,7 @@
         <v>0.5</v>
       </c>
       <c r="Z3" t="n">
-        <v>1588910166.938491</v>
+        <v>477083925.5524923</v>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
@@ -14675,79 +14675,79 @@
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AQ3" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AR3" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AS3" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AT3" t="n">
-        <v>22437895.17584041</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AU3" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AV3" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AW3" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AX3" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AY3" t="n">
-        <v>28362065.5938178</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AZ3" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BA3" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BB3" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BC3" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BD3" t="n">
-        <v>3895196.24798489</v>
+        <v>1298398.749328297</v>
       </c>
       <c r="BE3" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BF3" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BG3" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BH3" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BI3" t="n">
-        <v>4385488249.652888</v>
+        <v>1461829416.550962</v>
       </c>
       <c r="BJ3" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BK3" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BL3" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BM3" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BN3" t="n">
-        <v>2362801048.856053</v>
+        <v>787600349.6186843</v>
       </c>
       <c r="BO3" t="inlineStr"/>
       <c r="BP3" t="inlineStr"/>
@@ -15221,7 +15221,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.759712215371368e+16</v>
+        <v>2.463597101519915e+16</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
@@ -15246,7 +15246,7 @@
         <v>1000</v>
       </c>
       <c r="M2" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -15257,14 +15257,14 @@
         <v>0.3</v>
       </c>
       <c r="P2" t="n">
-        <v>3651970</v>
+        <v>3651985</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
         <v>2e+20</v>
       </c>
       <c r="S2" t="n">
-        <v>2.777777777777778e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -15283,7 +15283,7 @@
         <v>0.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>488808948.7142688</v>
+        <v>1026498792.299964</v>
       </c>
       <c r="AA2" t="n">
         <v>100</v>
@@ -15464,13 +15464,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2.794826622829694e+16</v>
+        <v>1.676895973697816e+16</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>6866650600.375151</v>
+        <v>3433325300.187575</v>
       </c>
       <c r="G3" t="n">
         <v>0.1472880275120053</v>
@@ -15486,10 +15486,10 @@
         <v>20</v>
       </c>
       <c r="L3" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="M3" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -15500,7 +15500,7 @@
         <v>0.4</v>
       </c>
       <c r="P3" t="n">
-        <v>2901117</v>
+        <v>1902924</v>
       </c>
       <c r="Q3" t="n">
         <v>2.696979113134065e+16</v>
@@ -15526,7 +15526,7 @@
         <v>4.5</v>
       </c>
       <c r="Z3" t="n">
-        <v>1552681457.127608</v>
+        <v>931608874.2765646</v>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
@@ -15544,64 +15544,64 @@
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AQ3" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AR3" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AS3" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AT3" t="n">
-        <v>14958596.78389361</v>
+        <v>7479298.391946803</v>
       </c>
       <c r="AU3" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AV3" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AW3" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AX3" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AY3" t="n">
-        <v>18908043.72921186</v>
+        <v>9454021.864605932</v>
       </c>
       <c r="AZ3" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BA3" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BB3" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BC3" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BD3" t="n">
-        <v>18673358.43440775</v>
+        <v>9336679.217203876</v>
       </c>
       <c r="BE3" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BF3" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BG3" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BH3" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BI3" t="n">
-        <v>356992075.1887032</v>
+        <v>178496037.5943516</v>
       </c>
       <c r="BJ3" t="n">
         <v>0</v>
@@ -16090,7 +16090,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3.113260860270707e+16</v>
+        <v>2.671953057464017e+16</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
@@ -16123,17 +16123,17 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="P2" t="n">
-        <v>3238540</v>
+        <v>3238507</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
         <v>2e+20</v>
       </c>
       <c r="S2" t="n">
-        <v>8.333333333333333e-08</v>
+        <v>1.111111111111111e-07</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -16152,7 +16152,7 @@
         <v>0.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>2594384050.225589</v>
+        <v>2968836730.515574</v>
       </c>
       <c r="AA2" t="n">
         <v>100</v>
@@ -16333,13 +16333,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3917755605130725</v>
+        <v>1.175326681539218e+17</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>434516298.6625866</v>
+        <v>8690325973.251732</v>
       </c>
       <c r="G3" t="n">
         <v>0.0291640551121764</v>
@@ -16355,10 +16355,10 @@
         <v>15</v>
       </c>
       <c r="L3" t="n">
-        <v>100</v>
+        <v>2000</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -16369,7 +16369,7 @@
         <v>0.3</v>
       </c>
       <c r="P3" t="n">
-        <v>523399</v>
+        <v>4515799</v>
       </c>
       <c r="Q3" t="n">
         <v>1.563254491497592e+16</v>
@@ -16378,7 +16378,7 @@
         <v>1.5e+20</v>
       </c>
       <c r="S3" t="n">
-        <v>5.555555555555555e-08</v>
+        <v>4.166666666666666e-08</v>
       </c>
       <c r="T3" t="b">
         <v>1</v>
@@ -16395,7 +16395,7 @@
         <v>1.5</v>
       </c>
       <c r="Z3" t="n">
-        <v>217653089.1739292</v>
+        <v>4897194506.413406</v>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
@@ -16413,64 +16413,64 @@
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AQ3" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AR3" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AS3" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AT3" t="n">
-        <v>866747.7855311844</v>
+        <v>17334955.71062369</v>
       </c>
       <c r="AU3" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AV3" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AW3" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AX3" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AY3" t="n">
-        <v>1075910.729652295</v>
+        <v>21518214.59304591</v>
       </c>
       <c r="AZ3" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BA3" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BB3" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BC3" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BD3" t="n">
-        <v>272803.9961756691</v>
+        <v>5456079.923513383</v>
       </c>
       <c r="BE3" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BF3" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BG3" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BH3" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BI3" t="n">
-        <v>75992794.19996466</v>
+        <v>1519855883.999293</v>
       </c>
       <c r="BJ3" t="n">
         <v>0</v>

</xml_diff>